<commit_message>
Correction des erreurs qa a9b64e7eff237859bb5e511219fec358368b7b7b
</commit_message>
<xml_diff>
--- a/qaFHIRErrors/ig/StructureDefinition-fr-advance-directive-document.xlsx
+++ b/qaFHIRErrors/ig/StructureDefinition-fr-advance-directive-document.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-19T10:06:59+00:00</t>
+    <t>2026-08-20T14:37:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1339,7 +1339,7 @@
     <t>Typical use of this is a Document code with class = CDA.</t>
   </si>
   <si>
-    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-type-directive-anticipee-cisis|20260619134043</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-type-directive-anticipee-cisis|20260716085853</t>
   </si>
   <si>
     <t>Consent.provision.dataPeriod</t>

</xml_diff>